<commit_message>
Update item mappings and parser support
</commit_message>
<xml_diff>
--- a/data/item和品名对应表.xlsx
+++ b/data/item和品名对应表.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michael/customs_doc_generator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65AAFF10-1695-814F-9D22-C9C4A08563DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70ED5F5-328C-BA46-BDE4-082BBBF32856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15800" yWindow="2040" windowWidth="28100" windowHeight="17360" xr2:uid="{91E03C8D-3782-F04D-A948-D1C2AEB1D78B}"/>
+    <workbookView xWindow="6100" yWindow="2040" windowWidth="28100" windowHeight="17360" xr2:uid="{91E03C8D-3782-F04D-A948-D1C2AEB1D78B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="OLE_LINK1" localSheetId="0">Sheet1!$C$27</definedName>
+    <definedName name="OLE_LINK1" localSheetId="0">Sheet1!$C$29</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="83">
   <si>
     <t>品名</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -467,6 +467,14 @@
   </si>
   <si>
     <t>机织|染色|平纹100%涤纶，幅宽1.45米，克重：g/m2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Buckle Bands</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Keychain</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -878,7 +886,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40FEC8A8-9350-734F-8D78-F41F50947005}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="34.6640625" customWidth="1"/>
@@ -943,339 +951,367 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="68">
+    <row r="5" spans="1:4" ht="102">
       <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>9113900090</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="68">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C5">
+      <c r="C6">
         <v>8708299000</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="102">
-      <c r="A6" t="s">
+    <row r="7" spans="1:4" ht="102">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>17</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>4202320000</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="136">
-      <c r="A7" t="s">
+    <row r="8" spans="1:4" ht="136">
+      <c r="A8" t="s">
         <v>19</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>20</v>
-      </c>
-      <c r="C7">
-        <v>9404909000</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="119">
-      <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
       </c>
       <c r="C8">
         <v>9404909000</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="119">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9">
+        <v>9404909000</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="136">
-      <c r="A9" t="s">
+    <row r="10" spans="1:4" ht="136">
+      <c r="A10" t="s">
         <v>25</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>26</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>4205009090</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="153">
-      <c r="A10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10">
-        <v>4202119090</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="153">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C11">
-        <v>4202190090</v>
+        <v>4202119090</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="153">
       <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12">
+        <v>4202190090</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="153">
+      <c r="A13" t="s">
         <v>34</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>35</v>
       </c>
-      <c r="C12">
+      <c r="C13">
         <v>4202119090</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="136">
-      <c r="A13" t="s">
+    <row r="14" spans="1:4" ht="136">
+      <c r="A14" t="s">
         <v>37</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B14" t="s">
         <v>38</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>4202220000</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="102">
-      <c r="A14" t="s">
+    <row r="15" spans="1:4" ht="102">
+      <c r="A15" t="s">
         <v>40</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>41</v>
       </c>
-      <c r="C14">
+      <c r="C15">
         <v>4202320000</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="68">
-      <c r="A15" t="s">
+    <row r="16" spans="1:4" ht="68">
+      <c r="A16" t="s">
         <v>43</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>44</v>
       </c>
-      <c r="C15">
+      <c r="C16">
         <v>3926909090</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="85">
-      <c r="A16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" t="s">
-        <v>47</v>
-      </c>
-      <c r="C16">
-        <v>4820100000</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="85">
       <c r="A17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17">
+        <v>4820100000</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="85">
+      <c r="A18" t="s">
         <v>49</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>50</v>
       </c>
-      <c r="C17">
+      <c r="C18">
         <v>4202320000</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="51">
-      <c r="A18" t="s">
-        <v>52</v>
-      </c>
-      <c r="B18" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18">
-        <v>4911101000</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="51">
       <c r="A19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19">
+        <v>4911101000</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="51">
+      <c r="A20" t="s">
         <v>55</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>56</v>
       </c>
-      <c r="C19">
+      <c r="C20">
         <v>6307909000</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="68">
-      <c r="A20" t="s">
+    <row r="21" spans="1:4" ht="68">
+      <c r="A21" t="s">
         <v>71</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>72</v>
       </c>
-      <c r="C20">
+      <c r="C21">
         <v>4205009090</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="102">
-      <c r="A21" t="s">
+    <row r="22" spans="1:4" ht="68">
+      <c r="A22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22">
+        <v>4205009090</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="102">
+      <c r="A23" t="s">
         <v>67</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B23" t="s">
         <v>58</v>
       </c>
-      <c r="C21">
+      <c r="C23">
         <v>5603149000</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="102">
-      <c r="A22" s="3" t="s">
+    <row r="24" spans="1:4" ht="102">
+      <c r="A24" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C22" s="3">
+      <c r="C24" s="3">
         <v>5603149000</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D24" s="4" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="119">
-      <c r="A23" s="3" t="s">
+    <row r="25" spans="1:4" ht="119">
+      <c r="A25" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="3">
+      <c r="C25" s="3">
         <v>5903209000</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D25" s="4" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="51">
-      <c r="A24" t="s">
+    <row r="26" spans="1:4" ht="51">
+      <c r="A26" t="s">
         <v>66</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B26" t="s">
         <v>60</v>
       </c>
-      <c r="C24">
+      <c r="C26">
         <v>4107121090</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="85">
-      <c r="A25" s="2" t="s">
+    <row r="27" spans="1:4" ht="85">
+      <c r="A27" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B25" t="s">
-        <v>58</v>
-      </c>
-      <c r="C25">
-        <v>5112200000</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="17">
-      <c r="A26" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" t="s">
-        <v>58</v>
-      </c>
-      <c r="C26">
-        <v>5407520000</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="68">
-      <c r="A27" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="B27" t="s">
         <v>58</v>
       </c>
       <c r="C27">
+        <v>5112200000</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="17">
+      <c r="A28" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28">
+        <v>5407520000</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="68">
+      <c r="A29" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29">
         <v>5112190000</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D29" s="2" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="102">
-      <c r="A28" t="s">
+    <row r="30" spans="1:4" ht="102">
+      <c r="A30" t="s">
         <v>65</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B30" t="s">
         <v>63</v>
       </c>
-      <c r="C28">
+      <c r="C30">
         <v>5903209000</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D30" s="2" t="s">
         <v>64</v>
       </c>
     </row>

</xml_diff>